<commit_message>
荣誉嘉宾数据结构优化【GoH Data Structure Optimization】
以下代码行数如无特殊说明，指的都是游戏数据提取脚本。
Without specific explanation, the following code lines belong to Game Data Extraction Program.
1. 移除了去格式化的两个简述键，因为它们和未去格式化的简述完全相同。（第5632和5669行。）
Removed two de-formatted description keys, for they're same as the original descriptions. (Lines 5632 and 5669.)
2. 同一语言的原始详细信息和去格式化详细信息现在紧挨着，而不是中间被一个默认语言的原始详细信息隔开来。（第5669行。）
Raw detailed tooltip and de-formatted detailed tooltip are now next to each other, instead of being separated by the raw detailed tooltip of the default language. (Line 5669.)
游戏数据提取主数据框结构工作簿已同步这些更改。
The above changes have been synchronized in Game Data Extraction Main Dataframe Workbook.
</commit_message>
<xml_diff>
--- a/Game Data Extraction Main Dataframe Structure.xlsx
+++ b/Game Data Extraction Main Dataframe Structure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C015DD4D-2E02-4924-BA8F-72C64634F31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB69180-9B45-4B8A-86F9-35B5325578C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="11" activeTab="15" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6869" uniqueCount="3527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6865" uniqueCount="3523">
   <si>
     <t>key</t>
   </si>
@@ -12604,14 +12604,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>{1ff99d7f} {bff2f361}_content_zh_burn</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{1ff99d7f} {bff2f361}_content_en_burn</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>{1ff99d7f} {3b7aa707}_content_zh_burn</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -12624,12 +12616,6 @@
   </si>
   <si>
     <t>详细信息（英文/去格式化）</t>
-  </si>
-  <si>
-    <t>简述（中文/去格式化）</t>
-  </si>
-  <si>
-    <t>简述（英文/去格式化）</t>
   </si>
 </sst>
 </file>
@@ -20322,7 +20308,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECF611F9-13A5-4CF6-B8E3-E0A2C9AC1592}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="36.125" bestFit="1" customWidth="1"/>
@@ -20440,7 +20426,7 @@
       </c>
       <c r="E6" s="4"/>
       <c r="G6">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20458,7 +20444,7 @@
       </c>
       <c r="E7" s="4"/>
       <c r="G7">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20476,7 +20462,7 @@
       </c>
       <c r="E8" s="4"/>
       <c r="G8">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20568,13 +20554,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>3519</v>
+        <v>3512</v>
       </c>
       <c r="C15" t="s">
-        <v>3525</v>
+        <v>1148</v>
       </c>
       <c r="G15">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20582,13 +20568,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>3520</v>
+        <v>3513</v>
       </c>
       <c r="C16" t="s">
-        <v>3526</v>
+        <v>1152</v>
       </c>
       <c r="G16">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20596,13 +20582,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>3512</v>
+        <v>3519</v>
       </c>
       <c r="C17" t="s">
-        <v>1148</v>
+        <v>3521</v>
       </c>
       <c r="G17">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20610,46 +20596,18 @@
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>3513</v>
+        <v>3520</v>
       </c>
       <c r="C18" t="s">
-        <v>1152</v>
+        <v>3522</v>
       </c>
       <c r="G18">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A19">
-        <v>17</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>3521</v>
-      </c>
-      <c r="C19" t="s">
-        <v>3523</v>
-      </c>
-      <c r="G19">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A20">
-        <v>18</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>3522</v>
-      </c>
-      <c r="C20" t="s">
-        <v>3524</v>
-      </c>
-      <c r="G20">
-        <v>16</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G20">
-    <sortCondition ref="A1:A20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G18">
+    <sortCondition ref="A1:A18"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
角色基础属性键修复和装备锻造器说明文本转换优化【Character Base Stat Key Fix and Item Anvil Tooltip Transformation Optimization】
以下代码行数如无特殊说明，指的都是游戏数据提取脚本。
Without specific explanation, the following code lines belong to Game Data Extraction Program.
1. [CommunityDragon/Data@e6313cc]英雄和角色工作表的表头中的基础属性部分现在解析为实际字符串。（第3839行和游戏数据提取主数据框结构工作簿`champion_header`工作表B146:B160。）
Basic stat part of headers in Champion and Character sheets are now resolved as actual strings. (Line 3839 and B146:B160 in `champion_header` sheet in Game Data Extraction Main Dataframe Structure workbook.)
2. 装备锻造器的说明文本现在进行了格式化。（第5396～5399行。）
Formatted item anvil tooltips. (Lines 5396～5399.)
</commit_message>
<xml_diff>
--- a/Game Data Extraction Main Dataframe Structure.xlsx
+++ b/Game Data Extraction Main Dataframe Structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB69180-9B45-4B8A-86F9-35B5325578C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B131E8-8D2B-440F-AFDF-7C82A45ABE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="11" activeTab="15" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="5" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
   </bookViews>
   <sheets>
     <sheet name="gameModeMap_header" sheetId="4" r:id="rId1"/>
@@ -11716,66 +11716,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>{8662cf12} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{4d37af28} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{9eedebad} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{913157bb} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{4af40dc3} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{e2b5d80d} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ea6100d5} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{18956a21} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{33c0bf27} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{01262a25} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{e62d9d92} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{7bd4b298} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{836cc82a} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{4f89c991} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{b9f2b365} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>基础生命值</t>
   </si>
   <si>
@@ -11821,31 +11761,6 @@
     <t>成长攻击速度</t>
   </si>
   <si>
-    <t>primaryAbilityResource {726ee5cd} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>primaryAbilityResource {6216bf7b} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>primaryAbilityResource {b35aa769} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>primaryAbilityResource {3a509002} {b35aa769}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>secondaryAbilityResource {726ee5cd} {b35aa769}</t>
-  </si>
-  <si>
-    <t>secondaryAbilityResource {6216bf7b} {b35aa769}</t>
-  </si>
-  <si>
-    <t>secondaryAbilityResource {b35aa769} {b35aa769}</t>
-  </si>
-  <si>
     <t>OutputOrder1 (champion; before v16.5)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -12616,6 +12531,72 @@
   </si>
   <si>
     <t>详细信息（英文/去格式化）</t>
+  </si>
+  <si>
+    <t>baseHPModifiable baseValue</t>
+  </si>
+  <si>
+    <t>hpPerLevelModifiable baseValue</t>
+  </si>
+  <si>
+    <t>baseStaticHPRegenModifiable baseValue</t>
+  </si>
+  <si>
+    <t>hpRegenPerLevelModifiable baseValue</t>
+  </si>
+  <si>
+    <t>baseDamageModifiable baseValue</t>
+  </si>
+  <si>
+    <t>damagePerLevelModifiable baseValue</t>
+  </si>
+  <si>
+    <t>baseArmorModifiable baseValue</t>
+  </si>
+  <si>
+    <t>armorPerLevelModifiable baseValue</t>
+  </si>
+  <si>
+    <t>baseMR baseValue</t>
+  </si>
+  <si>
+    <t>{01262a25} baseValue</t>
+  </si>
+  <si>
+    <t>baseMoveSpeedModifiable baseValue</t>
+  </si>
+  <si>
+    <t>attackRangeModifiable baseValue</t>
+  </si>
+  <si>
+    <t>attackSpeedModifiable baseValue</t>
+  </si>
+  <si>
+    <t>attackSpeedRatioModifiable baseValue</t>
+  </si>
+  <si>
+    <t>attackSpeedPerLevelModifiable baseValue</t>
+  </si>
+  <si>
+    <t>primaryAbilityResource {726ee5cd} baseValue</t>
+  </si>
+  <si>
+    <t>primaryAbilityResource {6216bf7b} baseValue</t>
+  </si>
+  <si>
+    <t>primaryAbilityResource baseValue baseValue</t>
+  </si>
+  <si>
+    <t>primaryAbilityResource {3a509002} baseValue</t>
+  </si>
+  <si>
+    <t>secondaryAbilityResource {726ee5cd} baseValue</t>
+  </si>
+  <si>
+    <t>secondaryAbilityResource {6216bf7b} baseValue</t>
+  </si>
+  <si>
+    <t>secondaryAbilityResource baseValue baseValue</t>
   </si>
 </sst>
 </file>
@@ -16917,10 +16898,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3399</v>
+        <v>3377</v>
       </c>
       <c r="C3" t="s">
-        <v>3426</v>
+        <v>3404</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>22</v>
@@ -16934,10 +16915,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>3400</v>
+        <v>3378</v>
       </c>
       <c r="C4" t="s">
-        <v>3492</v>
+        <v>3470</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>22</v>
@@ -16954,10 +16935,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>3401</v>
+        <v>3379</v>
       </c>
       <c r="C5" t="s">
-        <v>3429</v>
+        <v>3407</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>22</v>
@@ -16974,10 +16955,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>3402</v>
+        <v>3380</v>
       </c>
       <c r="C6" t="s">
-        <v>3435</v>
+        <v>3413</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>22</v>
@@ -16994,10 +16975,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>3403</v>
+        <v>3381</v>
       </c>
       <c r="C7" t="s">
-        <v>3437</v>
+        <v>3415</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>22</v>
@@ -17014,10 +16995,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>3404</v>
+        <v>3382</v>
       </c>
       <c r="C8" t="s">
-        <v>3436</v>
+        <v>3414</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>22</v>
@@ -17034,10 +17015,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>3405</v>
+        <v>3383</v>
       </c>
       <c r="C9" t="s">
-        <v>3442</v>
+        <v>3420</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>22</v>
@@ -17054,10 +17035,10 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>3406</v>
+        <v>3384</v>
       </c>
       <c r="C10" t="s">
-        <v>3443</v>
+        <v>3421</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>22</v>
@@ -17074,10 +17055,10 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>3407</v>
+        <v>3385</v>
       </c>
       <c r="C11" t="s">
-        <v>3448</v>
+        <v>3426</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>22</v>
@@ -17097,10 +17078,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>3408</v>
+        <v>3386</v>
       </c>
       <c r="C12" t="s">
-        <v>3449</v>
+        <v>3427</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>22</v>
@@ -17120,10 +17101,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>3409</v>
+        <v>3387</v>
       </c>
       <c r="C13" t="s">
-        <v>3495</v>
+        <v>3473</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>22</v>
@@ -17140,10 +17121,10 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>3410</v>
+        <v>3388</v>
       </c>
       <c r="C14" t="s">
-        <v>3450</v>
+        <v>3428</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>22</v>
@@ -17163,10 +17144,10 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>3411</v>
+        <v>3389</v>
       </c>
       <c r="C15" t="s">
-        <v>3451</v>
+        <v>3429</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>22</v>
@@ -17183,10 +17164,10 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>3412</v>
+        <v>3390</v>
       </c>
       <c r="C16" t="s">
-        <v>3452</v>
+        <v>3430</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>22</v>
@@ -17203,10 +17184,10 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>3413</v>
+        <v>3391</v>
       </c>
       <c r="C17" t="s">
-        <v>3494</v>
+        <v>3472</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>22</v>
@@ -17223,10 +17204,10 @@
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>3414</v>
+        <v>3392</v>
       </c>
       <c r="C18" t="s">
-        <v>3455</v>
+        <v>3433</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>22</v>
@@ -17243,10 +17224,10 @@
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>3415</v>
+        <v>3393</v>
       </c>
       <c r="C19" t="s">
-        <v>3458</v>
+        <v>3436</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>22</v>
@@ -17263,10 +17244,10 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>3416</v>
+        <v>3394</v>
       </c>
       <c r="C20" t="s">
-        <v>3496</v>
+        <v>3474</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>22</v>
@@ -17283,10 +17264,10 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>3417</v>
+        <v>3395</v>
       </c>
       <c r="C21" t="s">
-        <v>3463</v>
+        <v>3441</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>22</v>
@@ -17303,10 +17284,10 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>3418</v>
+        <v>3396</v>
       </c>
       <c r="C22" t="s">
-        <v>3464</v>
+        <v>3442</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>22</v>
@@ -17323,10 +17304,10 @@
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>3419</v>
+        <v>3397</v>
       </c>
       <c r="C23" t="s">
-        <v>3465</v>
+        <v>3443</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>22</v>
@@ -17343,10 +17324,10 @@
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>3420</v>
+        <v>3398</v>
       </c>
       <c r="C24" t="s">
-        <v>3474</v>
+        <v>3452</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>22</v>
@@ -17363,10 +17344,10 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>3421</v>
+        <v>3399</v>
       </c>
       <c r="C25" t="s">
-        <v>3475</v>
+        <v>3453</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>22</v>
@@ -17383,10 +17364,10 @@
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>3422</v>
+        <v>3400</v>
       </c>
       <c r="C26" t="s">
-        <v>3476</v>
+        <v>3454</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>22</v>
@@ -17403,10 +17384,10 @@
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>3423</v>
+        <v>3401</v>
       </c>
       <c r="C27" t="s">
-        <v>3489</v>
+        <v>3467</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>22</v>
@@ -17426,10 +17407,10 @@
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>3424</v>
+        <v>3402</v>
       </c>
       <c r="C28" t="s">
-        <v>3490</v>
+        <v>3468</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>22</v>
@@ -17446,10 +17427,10 @@
         <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>3425</v>
+        <v>3403</v>
       </c>
       <c r="C29" t="s">
-        <v>3491</v>
+        <v>3469</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>22</v>
@@ -17466,10 +17447,10 @@
         <v>28</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>3493</v>
+        <v>3471</v>
       </c>
       <c r="C30" t="s">
-        <v>3428</v>
+        <v>3406</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>22</v>
@@ -17483,10 +17464,10 @@
         <v>29</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>3431</v>
+        <v>3409</v>
       </c>
       <c r="C31" t="s">
-        <v>3427</v>
+        <v>3405</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>22</v>
@@ -17500,10 +17481,10 @@
         <v>30</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>3430</v>
+        <v>3408</v>
       </c>
       <c r="C32" t="s">
-        <v>3433</v>
+        <v>3411</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>22</v>
@@ -17517,10 +17498,10 @@
         <v>31</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>3432</v>
+        <v>3410</v>
       </c>
       <c r="C33" t="s">
-        <v>3434</v>
+        <v>3412</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>22</v>
@@ -17534,10 +17515,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>3438</v>
+        <v>3416</v>
       </c>
       <c r="C34" t="s">
-        <v>3444</v>
+        <v>3422</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>22</v>
@@ -17551,10 +17532,10 @@
         <v>33</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>3439</v>
+        <v>3417</v>
       </c>
       <c r="C35" t="s">
-        <v>3445</v>
+        <v>3423</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>22</v>
@@ -17568,10 +17549,10 @@
         <v>34</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>3440</v>
+        <v>3418</v>
       </c>
       <c r="C36" t="s">
-        <v>3446</v>
+        <v>3424</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>22</v>
@@ -17585,10 +17566,10 @@
         <v>35</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>3441</v>
+        <v>3419</v>
       </c>
       <c r="C37" t="s">
-        <v>3447</v>
+        <v>3425</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>22</v>
@@ -17602,10 +17583,10 @@
         <v>36</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>3453</v>
+        <v>3431</v>
       </c>
       <c r="C38" t="s">
-        <v>3456</v>
+        <v>3434</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>22</v>
@@ -17619,10 +17600,10 @@
         <v>37</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>3454</v>
+        <v>3432</v>
       </c>
       <c r="C39" t="s">
-        <v>3457</v>
+        <v>3435</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>22</v>
@@ -17636,10 +17617,10 @@
         <v>38</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>3459</v>
+        <v>3437</v>
       </c>
       <c r="C40" t="s">
-        <v>3461</v>
+        <v>3439</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>22</v>
@@ -17653,10 +17634,10 @@
         <v>39</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>3460</v>
+        <v>3438</v>
       </c>
       <c r="C41" t="s">
-        <v>3462</v>
+        <v>3440</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>22</v>
@@ -17670,10 +17651,10 @@
         <v>40</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>3466</v>
+        <v>3444</v>
       </c>
       <c r="C42" t="s">
-        <v>3470</v>
+        <v>3448</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>22</v>
@@ -17687,10 +17668,10 @@
         <v>41</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>3467</v>
+        <v>3445</v>
       </c>
       <c r="C43" t="s">
-        <v>3471</v>
+        <v>3449</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>22</v>
@@ -17704,10 +17685,10 @@
         <v>42</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>3468</v>
+        <v>3446</v>
       </c>
       <c r="C44" t="s">
-        <v>3472</v>
+        <v>3450</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>22</v>
@@ -17721,10 +17702,10 @@
         <v>43</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>3469</v>
+        <v>3447</v>
       </c>
       <c r="C45" t="s">
-        <v>3473</v>
+        <v>3451</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>22</v>
@@ -17738,10 +17719,10 @@
         <v>44</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>3477</v>
+        <v>3455</v>
       </c>
       <c r="C46" t="s">
-        <v>3478</v>
+        <v>3456</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>22</v>
@@ -17755,10 +17736,10 @@
         <v>45</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>3479</v>
+        <v>3457</v>
       </c>
       <c r="C47" t="s">
-        <v>3480</v>
+        <v>3458</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>22</v>
@@ -17772,10 +17753,10 @@
         <v>46</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>3483</v>
+        <v>3461</v>
       </c>
       <c r="C48" t="s">
-        <v>3481</v>
+        <v>3459</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>22</v>
@@ -17789,10 +17770,10 @@
         <v>47</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>3484</v>
+        <v>3462</v>
       </c>
       <c r="C49" t="s">
-        <v>3482</v>
+        <v>3460</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>22</v>
@@ -17806,10 +17787,10 @@
         <v>48</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>3485</v>
+        <v>3463</v>
       </c>
       <c r="C50" t="s">
-        <v>3487</v>
+        <v>3465</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>22</v>
@@ -17823,10 +17804,10 @@
         <v>49</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>3486</v>
+        <v>3464</v>
       </c>
       <c r="C51" t="s">
-        <v>3488</v>
+        <v>3466</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>22</v>
@@ -20362,10 +20343,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3499</v>
+        <v>3477</v>
       </c>
       <c r="C3" t="s">
-        <v>3503</v>
+        <v>3481</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>22</v>
@@ -20380,10 +20361,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>3500</v>
+        <v>3478</v>
       </c>
       <c r="C4" t="s">
-        <v>3516</v>
+        <v>3494</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>22</v>
@@ -20398,7 +20379,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>3501</v>
+        <v>3479</v>
       </c>
       <c r="C5" t="s">
         <v>2891</v>
@@ -20416,7 +20397,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>3502</v>
+        <v>3480</v>
       </c>
       <c r="C6" t="s">
         <v>1082</v>
@@ -20434,10 +20415,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>3497</v>
+        <v>3475</v>
       </c>
       <c r="C7" t="s">
-        <v>3504</v>
+        <v>3482</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>22</v>
@@ -20452,10 +20433,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>3498</v>
+        <v>3476</v>
       </c>
       <c r="C8" t="s">
-        <v>3505</v>
+        <v>3483</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>22</v>
@@ -20470,10 +20451,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>3506</v>
+        <v>3484</v>
       </c>
       <c r="C9" t="s">
-        <v>3514</v>
+        <v>3492</v>
       </c>
       <c r="G9">
         <v>2</v>
@@ -20484,10 +20465,10 @@
         <v>8</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>3507</v>
+        <v>3485</v>
       </c>
       <c r="C10" t="s">
-        <v>3515</v>
+        <v>3493</v>
       </c>
       <c r="G10">
         <v>3</v>
@@ -20498,10 +20479,10 @@
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>3508</v>
+        <v>3486</v>
       </c>
       <c r="C11" t="s">
-        <v>3517</v>
+        <v>3495</v>
       </c>
       <c r="G11">
         <v>5</v>
@@ -20512,10 +20493,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>3509</v>
+        <v>3487</v>
       </c>
       <c r="C12" t="s">
-        <v>3518</v>
+        <v>3496</v>
       </c>
       <c r="G12">
         <v>6</v>
@@ -20526,7 +20507,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>3510</v>
+        <v>3488</v>
       </c>
       <c r="C13" t="s">
         <v>1547</v>
@@ -20540,7 +20521,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>3511</v>
+        <v>3489</v>
       </c>
       <c r="C14" t="s">
         <v>1548</v>
@@ -20554,7 +20535,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>3512</v>
+        <v>3490</v>
       </c>
       <c r="C15" t="s">
         <v>1148</v>
@@ -20568,7 +20549,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>3513</v>
+        <v>3491</v>
       </c>
       <c r="C16" t="s">
         <v>1152</v>
@@ -20582,10 +20563,10 @@
         <v>15</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>3519</v>
+        <v>3497</v>
       </c>
       <c r="C17" t="s">
-        <v>3521</v>
+        <v>3499</v>
       </c>
       <c r="G17">
         <v>12</v>
@@ -20596,10 +20577,10 @@
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>3520</v>
+        <v>3498</v>
       </c>
       <c r="C18" t="s">
-        <v>3522</v>
+        <v>3500</v>
       </c>
       <c r="G18">
         <v>14</v>
@@ -30362,16 +30343,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>3319</v>
+        <v>3297</v>
       </c>
       <c r="C5" t="s">
-        <v>3320</v>
+        <v>3298</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="G5">
         <v>19</v>
@@ -30382,16 +30363,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>3321</v>
+        <v>3299</v>
       </c>
       <c r="C6" t="s">
-        <v>3322</v>
+        <v>3300</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="G6">
         <v>20</v>
@@ -30402,16 +30383,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>3329</v>
+        <v>3307</v>
       </c>
       <c r="C7" t="s">
-        <v>3330</v>
+        <v>3308</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="F7" t="b">
         <v>0</v>
@@ -30425,16 +30406,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>3323</v>
+        <v>3301</v>
       </c>
       <c r="C8" t="s">
-        <v>3331</v>
+        <v>3309</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -30448,16 +30429,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>3325</v>
+        <v>3303</v>
       </c>
       <c r="C9" t="s">
-        <v>3326</v>
+        <v>3304</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="G9">
         <v>23</v>
@@ -30468,13 +30449,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>3327</v>
+        <v>3305</v>
       </c>
       <c r="C10" t="s">
-        <v>3328</v>
+        <v>3306</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E10" s="4"/>
       <c r="G10">
@@ -30504,13 +30485,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>3332</v>
+        <v>3310</v>
       </c>
       <c r="C12" t="s">
-        <v>3333</v>
+        <v>3311</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E12" s="4"/>
       <c r="G12">
@@ -30522,16 +30503,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>3334</v>
+        <v>3312</v>
       </c>
       <c r="C13" t="s">
-        <v>3335</v>
+        <v>3313</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="F13" t="b">
         <v>0</v>
@@ -30545,16 +30526,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>3336</v>
+        <v>3314</v>
       </c>
       <c r="C14" t="s">
-        <v>3337</v>
+        <v>3315</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
@@ -30568,13 +30549,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>3338</v>
+        <v>3316</v>
       </c>
       <c r="C15" t="s">
-        <v>3339</v>
+        <v>3317</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E15" s="4"/>
       <c r="G15">
@@ -30586,13 +30567,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>3340</v>
+        <v>3318</v>
       </c>
       <c r="C16" t="s">
-        <v>3341</v>
+        <v>3319</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E16" s="4"/>
       <c r="G16">
@@ -30604,13 +30585,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>3342</v>
+        <v>3320</v>
       </c>
       <c r="C17" t="s">
-        <v>3346</v>
+        <v>3324</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E17" s="4"/>
       <c r="G17">
@@ -30622,13 +30603,13 @@
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>3343</v>
+        <v>3321</v>
       </c>
       <c r="C18" t="s">
-        <v>3347</v>
+        <v>3325</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E18" s="4"/>
       <c r="G18">
@@ -30640,13 +30621,13 @@
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>3344</v>
+        <v>3322</v>
       </c>
       <c r="C19" t="s">
-        <v>3348</v>
+        <v>3326</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E19" s="4"/>
       <c r="G19">
@@ -30658,13 +30639,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>3360</v>
+        <v>3338</v>
       </c>
       <c r="C20" t="s">
-        <v>3361</v>
+        <v>3339</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E20" s="4"/>
       <c r="G20">
@@ -30676,13 +30657,13 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>3345</v>
+        <v>3323</v>
       </c>
       <c r="C21" t="s">
-        <v>3349</v>
+        <v>3327</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E21" s="4"/>
       <c r="G21">
@@ -30694,13 +30675,13 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C22" t="s">
-        <v>3351</v>
+        <v>3329</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E22" s="4"/>
       <c r="G22">
@@ -30712,16 +30693,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>3352</v>
+        <v>3330</v>
       </c>
       <c r="C23" t="s">
-        <v>3354</v>
+        <v>3332</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -30735,16 +30716,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>3353</v>
+        <v>3331</v>
       </c>
       <c r="C24" t="s">
-        <v>3355</v>
+        <v>3333</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="F24" t="b">
         <v>0</v>
@@ -30758,13 +30739,13 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>3356</v>
+        <v>3334</v>
       </c>
       <c r="C25" t="s">
-        <v>3359</v>
+        <v>3337</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" t="b">
@@ -30779,13 +30760,13 @@
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>3357</v>
+        <v>3335</v>
       </c>
       <c r="C26" t="s">
-        <v>3358</v>
+        <v>3336</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E26" s="4"/>
       <c r="G26">
@@ -30797,16 +30778,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>3362</v>
+        <v>3340</v>
       </c>
       <c r="C27" t="s">
-        <v>3364</v>
+        <v>3342</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="F27" t="b">
         <v>0</v>
@@ -30820,16 +30801,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>3363</v>
+        <v>3341</v>
       </c>
       <c r="C28" t="s">
-        <v>3365</v>
+        <v>3343</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
@@ -30843,13 +30824,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>3366</v>
+        <v>3344</v>
       </c>
       <c r="C29" t="s">
-        <v>3367</v>
+        <v>3345</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E29" s="4"/>
       <c r="G29">
@@ -30861,13 +30842,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>3368</v>
+        <v>3346</v>
       </c>
       <c r="C30" t="s">
-        <v>3369</v>
+        <v>3347</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" t="b">
@@ -30882,13 +30863,13 @@
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>3370</v>
+        <v>3348</v>
       </c>
       <c r="C31" t="s">
-        <v>3371</v>
+        <v>3349</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>3324</v>
+        <v>3302</v>
       </c>
       <c r="E31" s="4"/>
       <c r="G31">
@@ -30903,7 +30884,7 @@
         <v>888</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>3372</v>
+        <v>3350</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
@@ -30916,7 +30897,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>3373</v>
+        <v>3351</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>26</v>
@@ -30936,7 +30917,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>3374</v>
+        <v>3352</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>27</v>
@@ -30956,7 +30937,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>3375</v>
+        <v>3353</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>28</v>
@@ -30976,7 +30957,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>3376</v>
+        <v>3354</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>29</v>
@@ -30996,7 +30977,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>3377</v>
+        <v>3355</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>30</v>
@@ -31016,7 +30997,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>3378</v>
+        <v>3356</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>31</v>
@@ -31039,7 +31020,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>3379</v>
+        <v>3357</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>32</v>
@@ -31056,7 +31037,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>3380</v>
+        <v>3358</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>1308</v>
@@ -31074,7 +31055,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>3381</v>
+        <v>3359</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>1309</v>
@@ -31090,7 +31071,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>3382</v>
+        <v>3360</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>1310</v>
@@ -31108,7 +31089,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>3383</v>
+        <v>3361</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>1311</v>
@@ -31124,7 +31105,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>3384</v>
+        <v>3362</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>1312</v>
@@ -31142,7 +31123,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>3385</v>
+        <v>3363</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>1313</v>
@@ -34371,16 +34352,16 @@
         <v>881</v>
       </c>
       <c r="H1" t="s">
-        <v>3315</v>
+        <v>3293</v>
       </c>
       <c r="I1" t="s">
-        <v>3316</v>
+        <v>3294</v>
       </c>
       <c r="J1" t="s">
-        <v>3317</v>
+        <v>3295</v>
       </c>
       <c r="K1" t="s">
-        <v>3318</v>
+        <v>3296</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
@@ -38444,10 +38425,10 @@
         <v>144</v>
       </c>
       <c r="B146" s="3" t="s">
+        <v>3501</v>
+      </c>
+      <c r="C146" s="2" t="s">
         <v>3278</v>
-      </c>
-      <c r="C146" s="2" t="s">
-        <v>3293</v>
       </c>
       <c r="D146" s="4" t="s">
         <v>22</v>
@@ -38467,10 +38448,10 @@
         <v>145</v>
       </c>
       <c r="B147" s="3" t="s">
+        <v>3502</v>
+      </c>
+      <c r="C147" s="2" t="s">
         <v>3279</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>3294</v>
       </c>
       <c r="D147" s="4" t="s">
         <v>22</v>
@@ -38490,10 +38471,10 @@
         <v>146</v>
       </c>
       <c r="B148" s="3" t="s">
+        <v>3503</v>
+      </c>
+      <c r="C148" s="2" t="s">
         <v>3280</v>
-      </c>
-      <c r="C148" s="2" t="s">
-        <v>3295</v>
       </c>
       <c r="D148" s="4" t="s">
         <v>22</v>
@@ -38516,10 +38497,10 @@
         <v>147</v>
       </c>
       <c r="B149" s="3" t="s">
+        <v>3504</v>
+      </c>
+      <c r="C149" s="2" t="s">
         <v>3281</v>
-      </c>
-      <c r="C149" s="2" t="s">
-        <v>3296</v>
       </c>
       <c r="D149" s="4" t="s">
         <v>22</v>
@@ -38542,10 +38523,10 @@
         <v>148</v>
       </c>
       <c r="B150" s="3" t="s">
+        <v>3505</v>
+      </c>
+      <c r="C150" s="2" t="s">
         <v>3282</v>
-      </c>
-      <c r="C150" s="2" t="s">
-        <v>3297</v>
       </c>
       <c r="D150" s="4" t="s">
         <v>22</v>
@@ -38565,10 +38546,10 @@
         <v>149</v>
       </c>
       <c r="B151" s="3" t="s">
+        <v>3506</v>
+      </c>
+      <c r="C151" s="2" t="s">
         <v>3283</v>
-      </c>
-      <c r="C151" s="2" t="s">
-        <v>3298</v>
       </c>
       <c r="D151" s="4" t="s">
         <v>22</v>
@@ -38591,10 +38572,10 @@
         <v>150</v>
       </c>
       <c r="B152" s="3" t="s">
+        <v>3507</v>
+      </c>
+      <c r="C152" s="2" t="s">
         <v>3284</v>
-      </c>
-      <c r="C152" s="2" t="s">
-        <v>3299</v>
       </c>
       <c r="D152" s="4" t="s">
         <v>22</v>
@@ -38614,10 +38595,10 @@
         <v>151</v>
       </c>
       <c r="B153" s="3" t="s">
+        <v>3508</v>
+      </c>
+      <c r="C153" s="2" t="s">
         <v>3285</v>
-      </c>
-      <c r="C153" s="2" t="s">
-        <v>3300</v>
       </c>
       <c r="D153" s="4" t="s">
         <v>22</v>
@@ -38640,10 +38621,10 @@
         <v>152</v>
       </c>
       <c r="B154" s="3" t="s">
+        <v>3509</v>
+      </c>
+      <c r="C154" s="2" t="s">
         <v>3286</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>3301</v>
       </c>
       <c r="D154" s="4" t="s">
         <v>22</v>
@@ -38663,10 +38644,10 @@
         <v>153</v>
       </c>
       <c r="B155" s="3" t="s">
+        <v>3510</v>
+      </c>
+      <c r="C155" s="2" t="s">
         <v>3287</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>3302</v>
       </c>
       <c r="D155" s="4" t="s">
         <v>22</v>
@@ -38689,10 +38670,10 @@
         <v>154</v>
       </c>
       <c r="B156" s="3" t="s">
+        <v>3511</v>
+      </c>
+      <c r="C156" s="2" t="s">
         <v>3288</v>
-      </c>
-      <c r="C156" s="2" t="s">
-        <v>3303</v>
       </c>
       <c r="D156" s="4" t="s">
         <v>22</v>
@@ -38712,10 +38693,10 @@
         <v>155</v>
       </c>
       <c r="B157" s="3" t="s">
+        <v>3512</v>
+      </c>
+      <c r="C157" s="2" t="s">
         <v>3289</v>
-      </c>
-      <c r="C157" s="2" t="s">
-        <v>3304</v>
       </c>
       <c r="D157" s="4" t="s">
         <v>22</v>
@@ -38735,10 +38716,10 @@
         <v>156</v>
       </c>
       <c r="B158" s="3" t="s">
+        <v>3513</v>
+      </c>
+      <c r="C158" s="2" t="s">
         <v>3290</v>
-      </c>
-      <c r="C158" s="2" t="s">
-        <v>3305</v>
       </c>
       <c r="D158" s="4" t="s">
         <v>22</v>
@@ -38758,10 +38739,10 @@
         <v>157</v>
       </c>
       <c r="B159" s="3" t="s">
+        <v>3514</v>
+      </c>
+      <c r="C159" s="2" t="s">
         <v>3291</v>
-      </c>
-      <c r="C159" s="2" t="s">
-        <v>3306</v>
       </c>
       <c r="D159" s="4" t="s">
         <v>22</v>
@@ -38781,10 +38762,10 @@
         <v>158</v>
       </c>
       <c r="B160" s="3" t="s">
+        <v>3515</v>
+      </c>
+      <c r="C160" s="2" t="s">
         <v>3292</v>
-      </c>
-      <c r="C160" s="2" t="s">
-        <v>3307</v>
       </c>
       <c r="D160" s="4" t="s">
         <v>22</v>
@@ -39983,7 +39964,7 @@
         <v>198</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>3308</v>
+        <v>3516</v>
       </c>
       <c r="C200" s="2" t="s">
         <v>681</v>
@@ -40009,7 +39990,7 @@
         <v>199</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>3309</v>
+        <v>3517</v>
       </c>
       <c r="C201" s="2" t="s">
         <v>682</v>
@@ -40035,7 +40016,7 @@
         <v>200</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>3310</v>
+        <v>3518</v>
       </c>
       <c r="C202" s="2" t="s">
         <v>684</v>
@@ -40058,7 +40039,7 @@
         <v>201</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>3311</v>
+        <v>3519</v>
       </c>
       <c r="C203" s="2" t="s">
         <v>686</v>
@@ -40690,7 +40671,7 @@
         <v>221</v>
       </c>
       <c r="B223" s="14" t="s">
-        <v>3312</v>
+        <v>3520</v>
       </c>
       <c r="C223" s="13" t="s">
         <v>701</v>
@@ -40716,7 +40697,7 @@
         <v>222</v>
       </c>
       <c r="B224" s="14" t="s">
-        <v>3313</v>
+        <v>3521</v>
       </c>
       <c r="C224" s="13" t="s">
         <v>702</v>
@@ -40742,7 +40723,7 @@
         <v>223</v>
       </c>
       <c r="B225" s="14" t="s">
-        <v>3314</v>
+        <v>3522</v>
       </c>
       <c r="C225" s="13" t="s">
         <v>703</v>
@@ -53354,10 +53335,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3386</v>
+        <v>3364</v>
       </c>
       <c r="C3" t="s">
-        <v>3393</v>
+        <v>3371</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>22</v>
@@ -53372,10 +53353,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>3387</v>
+        <v>3365</v>
       </c>
       <c r="C4" t="s">
-        <v>3394</v>
+        <v>3372</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>22</v>
@@ -53392,10 +53373,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>3388</v>
+        <v>3366</v>
       </c>
       <c r="C5" t="s">
-        <v>3396</v>
+        <v>3374</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>22</v>
@@ -53412,10 +53393,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>3392</v>
+        <v>3370</v>
       </c>
       <c r="C6" t="s">
-        <v>3395</v>
+        <v>3373</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>22</v>
@@ -53432,10 +53413,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>3389</v>
+        <v>3367</v>
       </c>
       <c r="C7" t="s">
-        <v>3397</v>
+        <v>3375</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>22</v>
@@ -53452,7 +53433,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>3390</v>
+        <v>3368</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>22</v>
@@ -53472,10 +53453,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>3391</v>
+        <v>3369</v>
       </c>
       <c r="C9" t="s">
-        <v>3398</v>
+        <v>3376</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
斗魂竞技场强化符文数据框的逻辑值优化问题修复【Boolean Value Optimization BUG Fix in Arena Augment Dataframe】
修复了一个问题，该问题曾导致对可用性的逻辑值优化在提交5193856中被意外移除。
Fixed a BUG that caused the Boolean value optimization on "Enabled" was removed by accident in commit 5193856.
</commit_message>
<xml_diff>
--- a/Game Data Extraction Main Dataframe Structure.xlsx
+++ b/Game Data Extraction Main Dataframe Structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABEF8065-9495-4BBC-A4BC-C6A85EBA78A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9C789C-5A4F-4FBF-A2FC-414CD88B96F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2250" yWindow="1005" windowWidth="34725" windowHeight="18735" firstSheet="10" activeTab="13" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="10" activeTab="10" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
   </bookViews>
   <sheets>
     <sheet name="gameModeMap_header" sheetId="4" r:id="rId1"/>
@@ -18077,6 +18077,9 @@
       <c r="E4" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="F4" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="G4">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
字体数据整理支持【Font Data Organization Support】
现在，游戏数据提取脚本可以整理和导出字体数据。
Now, Game Data Extraction Program can organize and export font data.
表头模块中游戏数据提取部分添加了二级注释，分别对应各个选项。（表头模块第4574、4815、4873、5002、5617、5902、6065、6095、6124、6142和6173行。）
Level-2 comments are added into Header Module to correspond to each option of Game Data Extraction Program. (Lines 4574, 4815, 4873, 5002, 5617, 5902, 6065, 6095, 6124, 6142 and 6173 in Header Module.)
以下工作表已添加到游戏数据提取主数据框结构工作簿。
The following worksheets have been added into Game Data Extraction Program Main Dataframe Structure Workbook:
- `fontDesc_header`
- `fontType_header`
- `fontResolution_header`
- `fontStyle_header`
- `font_CSSStyle_header`
- `font_CSSIcon_header`
</commit_message>
<xml_diff>
--- a/Game Data Extraction Main Dataframe Structure.xlsx
+++ b/Game Data Extraction Main Dataframe Structure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8AA8B5-B45F-405F-9DAD-E36C8B787C08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8FF65B-8765-4B26-9217-24F2568E2396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3285" yWindow="2040" windowWidth="34725" windowHeight="18735" firstSheet="12" activeTab="16" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="37" activeTab="43" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
   </bookViews>
   <sheets>
     <sheet name="gameModeMap_header" sheetId="4" r:id="rId1"/>
@@ -51,6 +51,12 @@
     <sheet name="TFTPVENPC_header" sheetId="30" r:id="rId36"/>
     <sheet name="TFTScript_header" sheetId="26" r:id="rId37"/>
     <sheet name="TFTAnnouncement_header" sheetId="20" r:id="rId38"/>
+    <sheet name="fontDesc_header" sheetId="45" r:id="rId39"/>
+    <sheet name="fontType_header" sheetId="46" r:id="rId40"/>
+    <sheet name="fontResolution_header" sheetId="47" r:id="rId41"/>
+    <sheet name="fontStyle_header" sheetId="48" r:id="rId42"/>
+    <sheet name="font_CSSStyle_header" sheetId="50" r:id="rId43"/>
+    <sheet name="font_CSSIcon_header" sheetId="51" r:id="rId44"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">champion_spell_header!$A$1:$G$341</definedName>
@@ -76,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7140" uniqueCount="3648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7340" uniqueCount="3719">
   <si>
     <t>key</t>
   </si>
@@ -13075,6 +13081,290 @@
   </si>
   <si>
     <t>championName</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>typeData</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>resolutionData</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Color</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>shadowColor</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>outlineColor</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>glowColor</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SelectionBoxColor</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>colorblindColor</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>colorblindOutlineColor</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>fillTextureName</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>字体类型键</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>字体分辨率键</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>颜色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>轮廓颜色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>阴影颜色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>发光颜色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>选择框颜色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>色盲模式颜色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>色盲模式轮廓颜色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>填充纹理名称</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>localeName</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>mFontFilePath</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FontFilePathBold</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>语言</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>字体文件路径</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>粗体文件路径</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>autoScale</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>自动缩放</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>localeResolution_index</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>resolution_index</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>screenHeight</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>fontSize</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>outlineSize</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>shadowDepthX</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>shadowDepthY</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>分辨率语言方案序号</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>分辨率方案序号</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>屏幕高度</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>字体大小</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>轮廓大小</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>阴影横坐标</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>阴影纵坐标</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>displayName</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>variant displayName</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>variant {75000be4}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>variant WEIGHT</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>variant Style</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>变体显示名</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>变体文件路径</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>字体显示名</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>变体权重</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>变体样式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>variant_index</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>变体序号</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PathHashToSelf</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>tag</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>bold</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>italics</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>underline</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>路径检索字符串</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CSS样式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>加粗</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>斜体</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>下划线</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>修饰符标签</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>texture</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>纹理路径</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>纵坐标偏移量</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>localeType_index</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>语言配置类型序号</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>YAdjustment</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -34569,6 +34859,357 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78E52B18-32F2-44AB-BEB9-1A4D38FC3321}">
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>2699</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2775</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3648</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3658</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>3649</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3659</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>3650</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3660</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>3652</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3661</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>3655</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3665</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>3656</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3666</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>3651</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3662</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>3657</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3667</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>3653</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3663</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>3654</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3664</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B15" s="1"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B17" s="6"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B18" s="6"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B19" s="6"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B20" s="6"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="6"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B22" s="6"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="6"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B24" s="6"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B25" s="6"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B26" s="6"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B27" s="6"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B28" s="6"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B29" s="6"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F13">
+    <sortCondition ref="A1:A13"/>
+  </sortState>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F7F4C24-7612-49A7-BA2B-B3643B323BBD}">
   <sheetPr codeName="Sheet17"/>
@@ -35873,6 +36514,1401 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G86">
     <sortCondition ref="A1:A86"/>
   </sortState>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD168143-EF2F-4DA8-9552-0152D380A4CE}">
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="18.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3716</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3717</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3668</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3671</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>3669</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3672</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>3670</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3673</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B7" s="1"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="1"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B9" s="1"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B10" s="1"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B11" s="1"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B12" s="1"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B13" s="1"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B15" s="1"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B17" s="1"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B18" s="6"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B19" s="6"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B20" s="6"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="6"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B22" s="6"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="6"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B24" s="6"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B25" s="6"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B26" s="6"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B27" s="6"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B28" s="6"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B29" s="6"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+    </row>
+    <row r="30" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B30" s="6"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E0CB622-4366-4796-A425-D38A6B94B7C7}">
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>881</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="G2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3674</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3675</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>3676</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>3683</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="G4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>3668</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3671</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="15">
+        <v>4</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>3677</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>3684</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="G6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="15">
+        <v>5</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>3678</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>3685</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="15">
+        <v>6</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>3679</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>3686</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9" s="15">
+        <v>7</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>3680</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>3687</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="15">
+        <v>8</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>3681</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>3688</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A11" s="15">
+        <v>9</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>3682</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>3689</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B12" s="1"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B13" s="1"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B15" s="1"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B17" s="6"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B18" s="6"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B19" s="6"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B20" s="6"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="6"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B22" s="6"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="6"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B24" s="6"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B25" s="6"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B26" s="6"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B27" s="6"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B28" s="6"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B29" s="6"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B736A4E-0AE1-484F-B09E-E75E07B5469B}">
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3690</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3697</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>3700</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>3701</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>3691</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3695</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>3692</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>3696</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>3693</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>3698</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>3694</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>3699</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B9" s="1"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B10" s="1"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B11" s="1"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B12" s="1"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B13" s="1"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B15" s="1"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B17" s="1"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B18" s="6"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B19" s="6"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B20" s="6"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="6"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B22" s="6"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="6"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B24" s="6"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B25" s="6"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B26" s="6"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B27" s="6"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B28" s="6"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B29" s="6"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+    </row>
+    <row r="30" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B30" s="6"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F8">
+    <sortCondition ref="A1:A8"/>
+  </sortState>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D5E88C9-7DBC-4DF3-8CB1-5BAAF4537407}">
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>881</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="G2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3702</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3707</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="28">
+        <v>2</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>3703</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>3708</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="G4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>3650</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3660</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>3704</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>3709</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>3705</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>3710</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>3706</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>3711</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B9" s="1"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B10" s="1"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B11" s="1"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B12" s="1"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B13" s="1"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B15" s="1"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B17" s="1"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B18" s="6"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B19" s="6"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B20" s="6"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="6"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B22" s="6"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="6"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B24" s="6"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B25" s="6"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B26" s="6"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B27" s="6"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B28" s="6"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B29" s="6"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+    </row>
+    <row r="30" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B30" s="6"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C075FD25-724E-4851-9475-612792A0E498}">
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3702</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3707</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="28">
+        <v>2</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>3703</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>3712</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>3713</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3714</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>3718</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>3715</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B7" s="1"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="1"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B9" s="1"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B10" s="1"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B11" s="1"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B12" s="1"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B13" s="1"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B15" s="1"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B17" s="1"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B18" s="6"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B19" s="6"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B20" s="6"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="6"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B22" s="6"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="6"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B24" s="6"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B25" s="6"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B26" s="6"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B27" s="6"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B28" s="6"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B29" s="6"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+    </row>
+    <row r="30" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B30" s="6"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+    </row>
+  </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
云顶之弈赛季数据的逻辑值优化【Boolean Value Optimization of TFT Set Data】
修复了一个问题，该问题曾导致云顶之弈赛季数据表的一个字段没有进行逻辑值优化。
Fixed a BUG that caused a Boolean field in TFT set dataframe not to be optimized.
对应到游戏数据提取主数据框结构工作簿的TFTSet_header工作表F61单元格。
This corresponds to F61 cell in sheet `TFTSet_header` in Game Data Extraction Main Dataframe Workbook.
</commit_message>
<xml_diff>
--- a/Game Data Extraction Main Dataframe Structure.xlsx
+++ b/Game Data Extraction Main Dataframe Structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8FF65B-8765-4B26-9217-24F2568E2396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15431AEF-FB2C-4BE8-96AA-B65691EDCEF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="37" activeTab="43" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="20" activeTab="20" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
   </bookViews>
   <sheets>
     <sheet name="gameModeMap_header" sheetId="4" r:id="rId1"/>
@@ -24483,6 +24483,9 @@
       <c r="E61" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="F61" t="b">
+        <v>1</v>
+      </c>
       <c r="G61">
         <v>241</v>
       </c>

</xml_diff>

<commit_message>
强化符文数据框表头更新【Augment Dataframe Header Update】
1. 推测出了未解析的键的含义。（表头模块全部改动。）
Inferred the actual meaning of unresolved hashes. (All changes in Header Module.)
- “{ed593c9c}”键的含义是由16.10.774.9553版本对【精算风险】的一个BUG的修复发现的。
The meaning of "{ed593c9c}" key is determined by a BUG fix of Calculated Risk in v16.10.774.9553.
2. 调整了斗魂竞技场强化符文数据框的表头顺序。（游戏数据提取脚本全部改动。）
Adjusted the order of the header of Arena augment dataframe. (All changes in Game Data Extraction Program.)
</commit_message>
<xml_diff>
--- a/Game Data Extraction Main Dataframe Structure.xlsx
+++ b/Game Data Extraction Main Dataframe Structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15431AEF-FB2C-4BE8-96AA-B65691EDCEF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F184FE-15D1-4BE5-9056-A590C0AA2938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="20" activeTab="20" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="10" activeTab="10" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
   </bookViews>
   <sheets>
     <sheet name="gameModeMap_header" sheetId="4" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7340" uniqueCount="3719">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7343" uniqueCount="3721">
   <si>
     <t>key</t>
   </si>
@@ -13365,6 +13365,14 @@
   </si>
   <si>
     <t>YAdjustment</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>次级稀有度</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>不占用栏位</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -18774,7 +18782,7 @@
         <v>22</v>
       </c>
       <c r="G9">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -18794,7 +18802,7 @@
         <v>22</v>
       </c>
       <c r="G10">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -18909,6 +18917,9 @@
       <c r="B17" s="1" t="s">
         <v>3571</v>
       </c>
+      <c r="C17" t="s">
+        <v>3719</v>
+      </c>
       <c r="D17" s="4" t="s">
         <v>3572</v>
       </c>
@@ -18916,7 +18927,7 @@
         <v>3572</v>
       </c>
       <c r="G17">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -18933,7 +18944,7 @@
         <v>22</v>
       </c>
       <c r="G18">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -18963,6 +18974,9 @@
       <c r="B20" s="1" t="s">
         <v>3273</v>
       </c>
+      <c r="C20" t="s">
+        <v>3720</v>
+      </c>
       <c r="D20" s="4" t="s">
         <v>3572</v>
       </c>
@@ -18973,7 +18987,7 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -19368,7 +19382,7 @@
         <v>463</v>
       </c>
       <c r="G48">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -19419,7 +19433,7 @@
         <v>3572</v>
       </c>
       <c r="G51">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -19850,7 +19864,7 @@
   <dimension ref="A1:G56"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="36.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.375" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="9" style="4"/>
@@ -20209,6 +20223,9 @@
       </c>
       <c r="B20" s="1" t="s">
         <v>3273</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3720</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
游戏数据提取脚本的海克斯大乱斗强化符文表格字段清理【ARAM: Mayhem Augment Table Field Clearing of Game Data Extraction Program】
从海克斯大乱斗强化符文表格中移除了满级说明文本相关字段，因为强化符文等级系统并不适用于海克斯大乱斗。（游戏数据提取脚本第6599行和游戏数据提取主数据框结构工作簿`KiwiAugment_header`工作表G43:G50区域。）
Removed max-level tooltip related fields from ARAM: Mayhem augment table, because augment leveling system doesn't apply to ARAM: Mayhem. (Line 6599 in Game Data Extraction Program and Area G43:G50 in Sheet `KiwiAugment_header` in Game Data Extraction Program.)
此外，调整了该表的一个字段的名称。（表头模块第6318行和游戏数据提取主数据框结构工作簿`KiwiAugment_header`工作表C66单元格。）
Besides, adjusted a field's name of this table. (Line 6318 in Header Module and Cell C66 in Sheet `KiwiAugment_header` in Game Data Extraction Program.)
</commit_message>
<xml_diff>
--- a/Game Data Extraction Main Dataframe Structure.xlsx
+++ b/Game Data Extraction Main Dataframe Structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DD499E-3EE2-463C-B67E-99CAE782A487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFA38324-AC6D-468F-82D3-EF20C3FA312D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2775" yWindow="2100" windowWidth="34725" windowHeight="18735" firstSheet="11" activeTab="14" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="11" activeTab="12" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
   </bookViews>
   <sheets>
     <sheet name="gameModeMap_header" sheetId="4" r:id="rId1"/>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7517" uniqueCount="3823">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7517" uniqueCount="3824">
   <si>
     <t>key</t>
   </si>
@@ -13772,6 +13772,10 @@
   </si>
   <si>
     <t>augment AugmentPlatformId</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>任务线相关强化符文</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -20414,7 +20418,7 @@
         <v>22</v>
       </c>
       <c r="G8">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20431,7 +20435,7 @@
         <v>22</v>
       </c>
       <c r="G9">
-        <v>58</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20524,9 +20528,6 @@
       <c r="D14" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G14">
-        <v>46</v>
-      </c>
     </row>
     <row r="15" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A15">
@@ -20541,9 +20542,6 @@
       <c r="D15" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G15">
-        <v>51</v>
-      </c>
     </row>
     <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A16">
@@ -20559,7 +20557,7 @@
         <v>22</v>
       </c>
       <c r="G16">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20576,7 +20574,7 @@
         <v>22</v>
       </c>
       <c r="G17">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20676,7 +20674,7 @@
         <v>3569</v>
       </c>
       <c r="G22">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20696,7 +20694,7 @@
         <v>22</v>
       </c>
       <c r="G23">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20984,9 +20982,6 @@
       <c r="C43" t="s">
         <v>3555</v>
       </c>
-      <c r="G43">
-        <v>47</v>
-      </c>
     </row>
     <row r="44" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A44">
@@ -20998,9 +20993,6 @@
       <c r="C44" t="s">
         <v>3556</v>
       </c>
-      <c r="G44">
-        <v>48</v>
-      </c>
     </row>
     <row r="45" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A45">
@@ -21012,9 +21004,6 @@
       <c r="C45" t="s">
         <v>3557</v>
       </c>
-      <c r="G45">
-        <v>49</v>
-      </c>
     </row>
     <row r="46" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A46">
@@ -21026,9 +21015,6 @@
       <c r="C46" t="s">
         <v>3558</v>
       </c>
-      <c r="G46">
-        <v>50</v>
-      </c>
     </row>
     <row r="47" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A47">
@@ -21040,9 +21026,6 @@
       <c r="C47" t="s">
         <v>3559</v>
       </c>
-      <c r="G47">
-        <v>52</v>
-      </c>
     </row>
     <row r="48" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A48">
@@ -21054,9 +21037,6 @@
       <c r="C48" t="s">
         <v>3560</v>
       </c>
-      <c r="G48">
-        <v>53</v>
-      </c>
     </row>
     <row r="49" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A49">
@@ -21068,9 +21048,6 @@
       <c r="C49" t="s">
         <v>3561</v>
       </c>
-      <c r="G49">
-        <v>54</v>
-      </c>
     </row>
     <row r="50" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A50">
@@ -21082,9 +21059,6 @@
       <c r="C50" t="s">
         <v>3562</v>
       </c>
-      <c r="G50">
-        <v>55</v>
-      </c>
     </row>
     <row r="51" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A51">
@@ -21134,7 +21108,7 @@
         <v>22</v>
       </c>
       <c r="G53">
-        <v>57</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21151,7 +21125,7 @@
         <v>22</v>
       </c>
       <c r="G54">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21210,7 +21184,7 @@
         <v>3569</v>
       </c>
       <c r="G58">
-        <v>63</v>
+        <v>53</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21287,7 +21261,7 @@
         <v>22</v>
       </c>
       <c r="G63">
-        <v>66</v>
+        <v>56</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21330,13 +21304,13 @@
         <v>3775</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>3780</v>
+        <v>3823</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>22</v>
       </c>
       <c r="G66">
-        <v>61</v>
+        <v>51</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="15" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
海克斯大乱斗任务线字段更新【ARAM: Mayhem Questline Field Update】
跟进测试服16.13.786.2007版本的更新，向海克斯大乱斗任务线相关表头中添加了一个未知的逻辑值字段。
Following the update of PBE Patch 16.13.786.2007, added an unknown Boolean field into ARAM: Mayhem questline related headers.
添加了游戏数据提取主数据框结构工作簿的`KiwiAugment_header`工作表的第67行和`KiwiQuestline_header`工作表的第10行。
Added Line 67 in Sheet `KiwiAugment_header` and Line 10 in Sheet `KiwiQuestline_header` in Game Data Extraction Main Dataframe Structure Workbook.
</commit_message>
<xml_diff>
--- a/Game Data Extraction Main Dataframe Structure.xlsx
+++ b/Game Data Extraction Main Dataframe Structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFA38324-AC6D-468F-82D3-EF20C3FA312D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C3F841-24D4-4859-8B30-123A84A23C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="11" activeTab="12" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="11" activeTab="14" xr2:uid="{3B9B600D-37BF-42AF-A848-4C9EEE49C701}"/>
   </bookViews>
   <sheets>
     <sheet name="gameModeMap_header" sheetId="4" r:id="rId1"/>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7517" uniqueCount="3824">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7521" uniqueCount="3826">
   <si>
     <t>key</t>
   </si>
@@ -13776,6 +13776,14 @@
   </si>
   <si>
     <t>任务线相关强化符文</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>questline {c504ece0}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{c504ece0}</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -20264,7 +20272,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{889E42AC-5584-44B0-BFBD-399F3EB60349}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="53.875" bestFit="1" customWidth="1"/>
@@ -20384,7 +20392,7 @@
         <v>22</v>
       </c>
       <c r="G6">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20401,7 +20409,7 @@
         <v>22</v>
       </c>
       <c r="G7">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20418,7 +20426,7 @@
         <v>22</v>
       </c>
       <c r="G8">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20435,7 +20443,7 @@
         <v>22</v>
       </c>
       <c r="G9">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20492,7 +20500,7 @@
         <v>22</v>
       </c>
       <c r="G12">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20512,7 +20520,7 @@
         <v>22</v>
       </c>
       <c r="G13">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20557,7 +20565,7 @@
         <v>22</v>
       </c>
       <c r="G16">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20574,7 +20582,7 @@
         <v>22</v>
       </c>
       <c r="G17">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20674,7 +20682,7 @@
         <v>3569</v>
       </c>
       <c r="G22">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20694,7 +20702,7 @@
         <v>22</v>
       </c>
       <c r="G23">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20759,7 +20767,7 @@
         <v>476</v>
       </c>
       <c r="G27">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20773,7 +20781,7 @@
         <v>482</v>
       </c>
       <c r="G28">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20787,7 +20795,7 @@
         <v>477</v>
       </c>
       <c r="G29">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20801,7 +20809,7 @@
         <v>484</v>
       </c>
       <c r="G30">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20815,7 +20823,7 @@
         <v>478</v>
       </c>
       <c r="G31">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20829,7 +20837,7 @@
         <v>487</v>
       </c>
       <c r="G32">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20843,7 +20851,7 @@
         <v>473</v>
       </c>
       <c r="G33">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20857,7 +20865,7 @@
         <v>488</v>
       </c>
       <c r="G34">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20871,7 +20879,7 @@
         <v>3547</v>
       </c>
       <c r="G35">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20885,7 +20893,7 @@
         <v>3548</v>
       </c>
       <c r="G36">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20899,7 +20907,7 @@
         <v>3549</v>
       </c>
       <c r="G37">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20913,7 +20921,7 @@
         <v>3550</v>
       </c>
       <c r="G38">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20927,7 +20935,7 @@
         <v>3551</v>
       </c>
       <c r="G39">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20941,7 +20949,7 @@
         <v>3552</v>
       </c>
       <c r="G40">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20955,7 +20963,7 @@
         <v>3553</v>
       </c>
       <c r="G41">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -20969,7 +20977,7 @@
         <v>3554</v>
       </c>
       <c r="G42">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21108,7 +21116,7 @@
         <v>22</v>
       </c>
       <c r="G53">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21125,7 +21133,7 @@
         <v>22</v>
       </c>
       <c r="G54">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21184,7 +21192,7 @@
         <v>3569</v>
       </c>
       <c r="G58">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21244,7 +21252,7 @@
         <v>22</v>
       </c>
       <c r="G62">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21261,7 +21269,7 @@
         <v>22</v>
       </c>
       <c r="G63">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21310,18 +21318,25 @@
         <v>22</v>
       </c>
       <c r="G66">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A67" s="2">
         <v>65</v>
       </c>
-      <c r="B67" s="56" t="s">
-        <v>3782</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>3784</v>
+      <c r="B67" s="3" t="s">
+        <v>3824</v>
+      </c>
+      <c r="C67" s="2"/>
+      <c r="D67" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F67" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>21</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21329,10 +21344,10 @@
         <v>66</v>
       </c>
       <c r="B68" s="56" t="s">
-        <v>3783</v>
+        <v>3782</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>3785</v>
+        <v>3784</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21340,13 +21355,10 @@
         <v>67</v>
       </c>
       <c r="B69" s="56" t="s">
-        <v>3786</v>
+        <v>3783</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>3789</v>
-      </c>
-      <c r="G69">
-        <v>42</v>
+        <v>3785</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -21354,10 +21366,10 @@
         <v>68</v>
       </c>
       <c r="B70" s="56" t="s">
-        <v>3787</v>
+        <v>3786</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>3791</v>
+        <v>3789</v>
       </c>
       <c r="G70">
         <v>43</v>
@@ -21368,10 +21380,10 @@
         <v>69</v>
       </c>
       <c r="B71" s="56" t="s">
-        <v>3792</v>
+        <v>3787</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>3795</v>
+        <v>3791</v>
       </c>
       <c r="G71">
         <v>44</v>
@@ -21382,18 +21394,32 @@
         <v>70</v>
       </c>
       <c r="B72" s="56" t="s">
-        <v>3793</v>
+        <v>3792</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>3797</v>
+        <v>3795</v>
       </c>
       <c r="G72">
         <v>45</v>
       </c>
     </row>
+    <row r="73" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A73" s="2">
+        <v>71</v>
+      </c>
+      <c r="B73" s="56" t="s">
+        <v>3793</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>3797</v>
+      </c>
+      <c r="G73">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G72">
-    <sortCondition ref="A1:A72"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G73">
+    <sortCondition ref="A1:A73"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21926,7 +21952,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD2F21B-D8AF-420D-A08D-54B532589448}">
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="40.5" bestFit="1" customWidth="1"/>
@@ -22096,17 +22122,15 @@
       <c r="A10">
         <v>8</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>3802</v>
-      </c>
-      <c r="C10" t="s">
-        <v>3805</v>
-      </c>
-      <c r="D10" s="4"/>
+      <c r="B10" s="1" t="s">
+        <v>3825</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10">
-        <v>4</v>
+      <c r="F10" s="4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -22114,16 +22138,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>3803</v>
+        <v>3802</v>
       </c>
       <c r="C11" t="s">
-        <v>3806</v>
+        <v>3805</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -22131,24 +22155,27 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>3818</v>
+        <v>3803</v>
       </c>
       <c r="C12" t="s">
-        <v>3788</v>
+        <v>3806</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
+      <c r="G12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>3819</v>
+        <v>3818</v>
       </c>
       <c r="C13" t="s">
-        <v>3790</v>
+        <v>3788</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
@@ -22159,10 +22186,10 @@
         <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>3820</v>
+        <v>3819</v>
       </c>
       <c r="C14" t="s">
-        <v>3794</v>
+        <v>3790</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
@@ -22173,43 +22200,38 @@
         <v>13</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>3821</v>
+        <v>3820</v>
       </c>
       <c r="C15" t="s">
-        <v>3796</v>
+        <v>3794</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
+      <c r="A16">
         <v>14</v>
       </c>
-      <c r="B16" s="56" t="s">
-        <v>3799</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>3809</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>22</v>
-      </c>
+      <c r="B16" s="6" t="s">
+        <v>3821</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3796</v>
+      </c>
+      <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
-      <c r="G16">
-        <v>6</v>
-      </c>
     </row>
     <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>3800</v>
+      <c r="B17" s="56" t="s">
+        <v>3799</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>3810</v>
+        <v>3809</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>22</v>
@@ -22217,7 +22239,7 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -22225,10 +22247,10 @@
         <v>16</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>3801</v>
+        <v>3800</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>3817</v>
+        <v>3810</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>22</v>
@@ -22236,24 +22258,26 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B19" s="56" t="s">
-        <v>3807</v>
+      <c r="B19" s="3" t="s">
+        <v>3801</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>3811</v>
-      </c>
-      <c r="D19" s="4"/>
+        <v>3817</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -22261,16 +22285,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="56" t="s">
-        <v>3812</v>
+        <v>3807</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>3813</v>
+        <v>3811</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -22278,16 +22302,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="56" t="s">
-        <v>3808</v>
+        <v>3812</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>3815</v>
+        <v>3813</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -22295,42 +22319,53 @@
         <v>20</v>
       </c>
       <c r="B22" s="56" t="s">
-        <v>3814</v>
+        <v>3808</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>3816</v>
+        <v>3815</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A23" s="7">
+      <c r="A23" s="2">
         <v>21</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>3822</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>464</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>22</v>
-      </c>
+      <c r="B23" s="56" t="s">
+        <v>3814</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>3816</v>
+      </c>
+      <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B24" s="6"/>
-      <c r="D24" s="4"/>
+      <c r="A24" s="7">
+        <v>22</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>3822</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
+      <c r="G24">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B25" s="6"/>
@@ -22417,13 +22452,13 @@
       <c r="F38" s="4"/>
     </row>
     <row r="39" spans="2:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="B39" s="1"/>
+      <c r="B39" s="6"/>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
     </row>
     <row r="40" spans="2:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="B40" s="6"/>
+      <c r="B40" s="1"/>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
@@ -22470,9 +22505,15 @@
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
     </row>
+    <row r="48" spans="2:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="B48" s="6"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G23">
-    <sortCondition ref="A1:A23"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G24">
+    <sortCondition ref="A1:A24"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>